<commit_message>
Add comments to patch script
</commit_message>
<xml_diff>
--- a/events/2026/config/motions-ids.xlsx
+++ b/events/2026/config/motions-ids.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\projects\work\wsw-results\events\2026\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E73A60A-F035-4671-B120-F6FB21145667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758D61B0-4B8F-4FBD-B0D0-43E23F450EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="motions" sheetId="1" r:id="rId1"/>
@@ -1237,6 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:U86"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1491,7 +1492,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>16</v>
       </c>
@@ -1543,7 +1544,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>17</v>
       </c>
@@ -1656,7 +1657,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>19</v>
       </c>
@@ -1711,7 +1712,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>20</v>
       </c>
@@ -1769,7 +1770,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>21</v>
       </c>
@@ -1882,7 +1883,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>23</v>
       </c>
@@ -1937,7 +1938,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>24</v>
       </c>
@@ -1992,7 +1993,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>25</v>
       </c>
@@ -2105,7 +2106,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>27</v>
       </c>
@@ -2160,7 +2161,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>28</v>
       </c>
@@ -2215,7 +2216,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>29</v>
       </c>
@@ -2328,7 +2329,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>31</v>
       </c>
@@ -2383,7 +2384,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>32</v>
       </c>
@@ -2554,7 +2555,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>35</v>
       </c>
@@ -2667,7 +2668,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>37</v>
       </c>
@@ -2722,7 +2723,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>38</v>
       </c>
@@ -2777,7 +2778,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>39</v>
       </c>
@@ -2836,7 +2837,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>40</v>
       </c>
@@ -2891,7 +2892,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>41</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>42</v>
       </c>
@@ -3001,7 +3002,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>43</v>
       </c>
@@ -3114,7 +3115,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>45</v>
       </c>
@@ -3227,7 +3228,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>47</v>
       </c>
@@ -3286,7 +3287,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>48</v>
       </c>
@@ -3341,7 +3342,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>49</v>
       </c>
@@ -3396,7 +3397,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>50</v>
       </c>
@@ -3451,7 +3452,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>51</v>
       </c>
@@ -3506,7 +3507,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>52</v>
       </c>
@@ -3561,7 +3562,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>53</v>
       </c>
@@ -3616,7 +3617,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>54</v>
       </c>
@@ -3671,7 +3672,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>55</v>
       </c>
@@ -3843,7 +3844,7 @@
         <v>Motion 1641</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>58</v>
       </c>
@@ -3898,7 +3899,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>59</v>
       </c>
@@ -3953,7 +3954,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>60</v>
       </c>
@@ -4008,7 +4009,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>61</v>
       </c>
@@ -4060,7 +4061,7 @@
         <v>Motion 618</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>63</v>
       </c>
@@ -4118,7 +4119,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>64</v>
       </c>
@@ -4173,7 +4174,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>65</v>
       </c>
@@ -4228,7 +4229,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>66</v>
       </c>
@@ -4402,7 +4403,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>69</v>
       </c>
@@ -4515,7 +4516,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>71</v>
       </c>
@@ -4574,7 +4575,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>72</v>
       </c>
@@ -4687,7 +4688,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>75</v>
       </c>
@@ -4742,7 +4743,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>76</v>
       </c>
@@ -4797,7 +4798,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>77</v>
       </c>
@@ -4849,7 +4850,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>78</v>
       </c>
@@ -4904,7 +4905,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>79</v>
       </c>
@@ -4959,7 +4960,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>80</v>
       </c>
@@ -5014,7 +5015,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>81</v>
       </c>
@@ -5072,7 +5073,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>82</v>
       </c>
@@ -5188,7 +5189,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>84</v>
       </c>
@@ -5240,7 +5241,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>85</v>
       </c>
@@ -5353,7 +5354,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>87</v>
       </c>
@@ -5408,7 +5409,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>88</v>
       </c>
@@ -5467,7 +5468,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>89</v>
       </c>
@@ -5522,7 +5523,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>90</v>
       </c>
@@ -5580,7 +5581,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>91</v>
       </c>
@@ -5639,7 +5640,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>92</v>
       </c>
@@ -5691,7 +5692,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>93</v>
       </c>
@@ -5750,7 +5751,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>94</v>
       </c>
@@ -5863,7 +5864,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>97</v>
       </c>
@@ -5921,7 +5922,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>98</v>
       </c>
@@ -6034,7 +6035,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>100</v>
       </c>
@@ -6093,7 +6094,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U86" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:U86" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="13">
+      <filters>
+        <filter val="2"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
Add details for buoys
</commit_message>
<xml_diff>
--- a/events/2026/config/motions-ids.xlsx
+++ b/events/2026/config/motions-ids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mike\projects\work\wsw-results\events\2026\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758D61B0-4B8F-4FBD-B0D0-43E23F450EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA0B88F-99CD-4B16-9EBC-2226B3933F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1237,7 +1237,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:U86"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1492,7 +1491,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>16</v>
       </c>
@@ -1544,7 +1543,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>17</v>
       </c>
@@ -1657,7 +1656,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>19</v>
       </c>
@@ -1712,7 +1711,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>20</v>
       </c>
@@ -1770,7 +1769,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>21</v>
       </c>
@@ -1883,7 +1882,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>23</v>
       </c>
@@ -1938,7 +1937,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>24</v>
       </c>
@@ -1993,7 +1992,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>25</v>
       </c>
@@ -2106,7 +2105,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>27</v>
       </c>
@@ -2161,7 +2160,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>28</v>
       </c>
@@ -2216,7 +2215,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>29</v>
       </c>
@@ -2329,7 +2328,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>31</v>
       </c>
@@ -2384,7 +2383,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>32</v>
       </c>
@@ -2555,7 +2554,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>35</v>
       </c>
@@ -2668,7 +2667,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>37</v>
       </c>
@@ -2723,7 +2722,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>38</v>
       </c>
@@ -2778,7 +2777,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>39</v>
       </c>
@@ -2837,7 +2836,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>40</v>
       </c>
@@ -2892,7 +2891,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>41</v>
       </c>
@@ -2947,7 +2946,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>42</v>
       </c>
@@ -3002,7 +3001,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>43</v>
       </c>
@@ -3115,7 +3114,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>45</v>
       </c>
@@ -3228,7 +3227,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>47</v>
       </c>
@@ -3287,7 +3286,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>48</v>
       </c>
@@ -3342,7 +3341,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>49</v>
       </c>
@@ -3397,7 +3396,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>50</v>
       </c>
@@ -3452,7 +3451,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>51</v>
       </c>
@@ -3507,7 +3506,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>52</v>
       </c>
@@ -3562,7 +3561,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>53</v>
       </c>
@@ -3617,7 +3616,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>54</v>
       </c>
@@ -3672,7 +3671,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>55</v>
       </c>
@@ -3844,7 +3843,7 @@
         <v>Motion 1641</v>
       </c>
     </row>
-    <row r="47" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>58</v>
       </c>
@@ -3899,7 +3898,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>59</v>
       </c>
@@ -3954,7 +3953,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>60</v>
       </c>
@@ -4009,7 +4008,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>61</v>
       </c>
@@ -4061,7 +4060,7 @@
         <v>Motion 618</v>
       </c>
     </row>
-    <row r="51" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>63</v>
       </c>
@@ -4119,7 +4118,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>64</v>
       </c>
@@ -4174,7 +4173,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>65</v>
       </c>
@@ -4229,7 +4228,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>66</v>
       </c>
@@ -4403,7 +4402,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>69</v>
       </c>
@@ -4516,7 +4515,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>71</v>
       </c>
@@ -4575,7 +4574,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>72</v>
       </c>
@@ -4688,7 +4687,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>75</v>
       </c>
@@ -4743,7 +4742,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>76</v>
       </c>
@@ -4798,7 +4797,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>77</v>
       </c>
@@ -4850,7 +4849,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>78</v>
       </c>
@@ -4905,7 +4904,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>79</v>
       </c>
@@ -4960,7 +4959,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>80</v>
       </c>
@@ -5015,7 +5014,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>81</v>
       </c>
@@ -5073,7 +5072,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>82</v>
       </c>
@@ -5189,7 +5188,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>84</v>
       </c>
@@ -5241,7 +5240,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>85</v>
       </c>
@@ -5354,7 +5353,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>87</v>
       </c>
@@ -5409,7 +5408,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>88</v>
       </c>
@@ -5468,7 +5467,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>89</v>
       </c>
@@ -5523,7 +5522,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>90</v>
       </c>
@@ -5581,7 +5580,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>91</v>
       </c>
@@ -5640,7 +5639,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>92</v>
       </c>
@@ -5692,7 +5691,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>93</v>
       </c>
@@ -5751,7 +5750,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>94</v>
       </c>
@@ -5864,7 +5863,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>97</v>
       </c>
@@ -5922,7 +5921,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>98</v>
       </c>
@@ -6035,7 +6034,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>100</v>
       </c>
@@ -6094,13 +6093,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U86" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="13">
-      <filters>
-        <filter val="2"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:U86" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>